<commit_message>
Extend Student model with parent/ethnicity/birth/ID fields, full mock data
</commit_message>
<xml_diff>
--- a/七（4）班学生信息_模拟数据.xlsx
+++ b/七（4）班学生信息_模拟数据.xlsx
@@ -952,30 +952,30 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>410422201301213847</t>
+          <t>410422201210233847</t>
         </is>
       </c>
       <c r="G4" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>朱宇健</t>
+          <t>韩杰</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>13855940781</t>
+          <t>18394078161</t>
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>韩艳</t>
+          <t>傅燕</t>
         </is>
       </c>
       <c r="K4" s="14" t="inlineStr">
@@ -1010,12 +1010,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>410422201307236805</t>
+          <t>410422201303013712</t>
         </is>
       </c>
       <c r="G5" s="13" t="n">
@@ -1023,27 +1023,27 @@
       </c>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>谢平</t>
+          <t>郭洋</t>
         </is>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
-          <t>15141928327</t>
+          <t>15083276483</t>
         </is>
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>韩玉</t>
+          <t>梁静敏</t>
         </is>
       </c>
       <c r="K5" s="14" t="inlineStr">
         <is>
-          <t>19935030564</t>
+          <t>18264139537</t>
         </is>
       </c>
       <c r="L5" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-保安镇水郭村936号</t>
+          <t>河南省-平顶山市-叶县-田庄乡王庄村147号</t>
         </is>
       </c>
     </row>
@@ -1068,40 +1068,40 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>2012年12月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>410422201212184909</t>
+          <t>410422201301138381</t>
         </is>
       </c>
       <c r="G6" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>曹俊</t>
+          <t>曾阳</t>
         </is>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>18824238849</t>
+          <t>18653287101</t>
         </is>
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>于悦</t>
+          <t>吴巧</t>
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
-          <t>13987101226</t>
+          <t>18791669784</t>
         </is>
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡盆杨村395号</t>
+          <t>河南省-平顶山市-叶县-邓李乡小张庄697号</t>
         </is>
       </c>
     </row>
@@ -1126,12 +1126,12 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>410422201304288978</t>
+          <t>410422201301151593</t>
         </is>
       </c>
       <c r="G7" s="13" t="n">
@@ -1139,27 +1139,27 @@
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>何伟</t>
+          <t>宋涛平</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
-          <t>13884514627</t>
+          <t>18804828148</t>
         </is>
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>王玲</t>
+          <t>彭英巧</t>
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr">
         <is>
-          <t>15081489325</t>
+          <t>19980957015</t>
         </is>
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇老鸦张村553号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡凤岭新村246号</t>
         </is>
       </c>
     </row>
@@ -1184,40 +1184,40 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年07月</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>41042220120901787X</t>
+          <t>410422201307084381</t>
         </is>
       </c>
       <c r="G8" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>梁然凯</t>
+          <t>朱哲</t>
         </is>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
-          <t>15930391171</t>
+          <t>15146578713</t>
         </is>
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>许秀英萱</t>
+          <t>高丽</t>
         </is>
       </c>
       <c r="K8" s="14" t="inlineStr">
         <is>
-          <t>19924896383</t>
+          <t>19939301031</t>
         </is>
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡凤岭新村409号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡孟庄村881号</t>
         </is>
       </c>
     </row>
@@ -1242,40 +1242,40 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>410422201303115843</t>
+          <t>410422201212199951</t>
         </is>
       </c>
       <c r="G9" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>邓晨辉</t>
+          <t>周豪豪</t>
         </is>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
-          <t>13750983930</t>
+          <t>18731165667</t>
         </is>
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>陈静敏</t>
+          <t>刘娟婷</t>
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr">
         <is>
-          <t>18218347382</t>
+          <t>13833387262</t>
         </is>
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡孙庄村591号</t>
+          <t>河南省-平顶山市-叶县-常村镇王庄村256号</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1300,12 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>41042220130501151X</t>
+          <t>410422201306098538</t>
         </is>
       </c>
       <c r="G10" s="13" t="n">
@@ -1313,27 +1313,27 @@
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>冯建华阳</t>
+          <t>刘哲</t>
         </is>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
-          <t>18366701065</t>
+          <t>13732677360</t>
         </is>
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>赵红晴</t>
+          <t>徐佳佳</t>
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr">
         <is>
-          <t>18826247317</t>
+          <t>15874687234</t>
         </is>
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇陈庄村101号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡孟庄村594号</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>410422201306048538</t>
+          <t>41042220130627787X</t>
         </is>
       </c>
       <c r="G11" s="13" t="n">
@@ -1371,27 +1371,27 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>王勇</t>
+          <t>袁睿轩</t>
         </is>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
-          <t>15226773602</t>
+          <t>13721913619</t>
         </is>
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>韩芳</t>
+          <t>林敏</t>
         </is>
       </c>
       <c r="K11" s="14" t="inlineStr">
         <is>
-          <t>15874687234</t>
+          <t>18799854353</t>
         </is>
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡孟庄村594号</t>
+          <t>河南省-平顶山市-叶县-常村镇段庄村135号</t>
         </is>
       </c>
     </row>
@@ -1416,12 +1416,12 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>410422201210023673</t>
+          <t>410422201209053784</t>
         </is>
       </c>
       <c r="G12" s="13" t="n">
@@ -1429,27 +1429,27 @@
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>梁军豪</t>
+          <t>吕杰文</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>17782081219</t>
+          <t>17742513542</t>
         </is>
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>陈红</t>
+          <t>董晴</t>
         </is>
       </c>
       <c r="K12" s="14" t="inlineStr">
         <is>
-          <t>15299091699</t>
+          <t>17708412411</t>
         </is>
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-邓李乡杨岭庄村958号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡陈庄村160号</t>
         </is>
       </c>
     </row>
@@ -1474,40 +1474,40 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>41042220130809926X</t>
+          <t>410422201212145402</t>
         </is>
       </c>
       <c r="G13" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>梁鹏明</t>
+          <t>何轩</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
-          <t>15975107991</t>
+          <t>13616400524</t>
         </is>
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>陈晴玲</t>
+          <t>徐诗</t>
         </is>
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>13951354278</t>
+          <t>18780112805</t>
         </is>
       </c>
       <c r="L13" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡凤岭新村627号</t>
+          <t>河南省-平顶山市-叶县-水寨乡陈庄村152号</t>
         </is>
       </c>
     </row>
@@ -1532,12 +1532,12 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>410422201305298892</t>
+          <t>410422201303034123</t>
         </is>
       </c>
       <c r="G14" s="13" t="n">
@@ -1545,27 +1545,27 @@
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>傅波</t>
+          <t>林杰</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>13824118244</t>
+          <t>19969232260</t>
         </is>
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>彭梅</t>
+          <t>孙婷</t>
         </is>
       </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>15148740164</t>
+          <t>18734216073</t>
         </is>
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇小张庄342号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡王庄村359号</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>410422201307249956</t>
+          <t>410422201303245460</t>
         </is>
       </c>
       <c r="G15" s="13" t="n">
@@ -1603,27 +1603,27 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>徐晨</t>
+          <t>郭洋</t>
         </is>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
-          <t>18780112805</t>
+          <t>15858685014</t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>曾曦秀英</t>
+          <t>孙玲瑶</t>
         </is>
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>13645053315</t>
+          <t>18356981693</t>
         </is>
       </c>
       <c r="L15" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇陈庄村906号</t>
+          <t>河南省-平顶山市-叶县-常村镇孟庄村726号</t>
         </is>
       </c>
     </row>
@@ -1648,12 +1648,12 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>410422201307154364</t>
+          <t>410422201308183933</t>
         </is>
       </c>
       <c r="G16" s="13" t="n">
@@ -1661,27 +1661,27 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>吴鹏</t>
+          <t>胡凯</t>
         </is>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
-          <t>15060256342</t>
+          <t>18295148465</t>
         </is>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>赵佳</t>
+          <t>唐燕</t>
         </is>
       </c>
       <c r="K16" s="14" t="inlineStr">
         <is>
-          <t>17633754330</t>
+          <t>15166299468</t>
         </is>
       </c>
       <c r="L16" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-廉村镇水郭村409号</t>
+          <t>河南省-平顶山市-叶县-任店镇小张庄312号</t>
         </is>
       </c>
     </row>
@@ -1706,40 +1706,40 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>410422201210065460</t>
+          <t>410422201308027449</t>
         </is>
       </c>
       <c r="G17" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>郭浩</t>
+          <t>萧晨</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t>18685014294</t>
+          <t>15187214895</t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>张娟</t>
+          <t>杨红</t>
         </is>
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>18356981693</t>
+          <t>15232003791</t>
         </is>
       </c>
       <c r="L17" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇孟庄村726号</t>
+          <t>河南省-平顶山市-叶县-龚店乡李庄村908号</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>410422201305251004</t>
+          <t>410422201305122627</t>
         </is>
       </c>
       <c r="G18" s="13" t="n">
@@ -1777,27 +1777,27 @@
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>许建华</t>
+          <t>林超</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>13759514846</t>
+          <t>13516328708</t>
         </is>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>梁悦</t>
+          <t>林霞</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>19923662994</t>
+          <t>18888957986</t>
         </is>
       </c>
       <c r="L18" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-田庄乡陈庄村854号</t>
+          <t>河南省-平顶山市-叶县-任店镇陈庄村457号</t>
         </is>
       </c>
     </row>
@@ -1822,12 +1822,12 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2013年07月</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>41042220130125524X</t>
+          <t>410422201307245306</t>
         </is>
       </c>
       <c r="G19" s="13" t="n">
@@ -1835,27 +1835,27 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>于斌</t>
+          <t>邓然</t>
         </is>
       </c>
       <c r="I19" s="14" t="inlineStr">
         <is>
-          <t>18838721489</t>
+          <t>15871434558</t>
         </is>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>宋艳</t>
+          <t>杨秀英佳</t>
         </is>
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>15243320037</t>
+          <t>13931665876</t>
         </is>
       </c>
       <c r="L19" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡盆杨村467号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇水郭村853号</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>410422201306229508</t>
+          <t>410422201306074345</t>
         </is>
       </c>
       <c r="G20" s="13" t="n">
@@ -1893,27 +1893,27 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>韩然</t>
+          <t>彭辉</t>
         </is>
       </c>
       <c r="I20" s="14" t="inlineStr">
         <is>
-          <t>13901632870</t>
+          <t>15867065627</t>
         </is>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>傅红</t>
+          <t>周晴悦</t>
         </is>
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>13872788957</t>
+          <t>13516272046</t>
         </is>
       </c>
       <c r="L20" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡刘庄村437号</t>
+          <t>河南省-平顶山市-叶县-夏李乡水郭村466号</t>
         </is>
       </c>
     </row>
@@ -1933,17 +1933,17 @@
       </c>
       <c r="D21" s="40" t="inlineStr">
         <is>
-          <t>蒙古族</t>
+          <t>汉</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>410422201304176557</t>
+          <t>410422201302274199</t>
         </is>
       </c>
       <c r="G21" s="13" t="n">
@@ -1951,27 +1951,27 @@
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>徐豪</t>
+          <t>陈磊</t>
         </is>
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>15248734714</t>
+          <t>15230923271</t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>林玉</t>
+          <t>沈梅</t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>19912236231</t>
+          <t>15852991241</t>
         </is>
       </c>
       <c r="L21" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-田庄乡李庄村339号</t>
+          <t>河南省-平顶山市-叶县-水寨乡小张庄952号</t>
         </is>
       </c>
     </row>
@@ -1996,12 +1996,12 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>410422201304012697</t>
+          <t>410422201303237664</t>
         </is>
       </c>
       <c r="G22" s="13" t="n">
@@ -2009,27 +2009,27 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>朱峰</t>
+          <t>胡洋</t>
         </is>
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>13596705466</t>
+          <t>15214919058</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>许晴</t>
+          <t>于怡婷</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>15273467065</t>
+          <t>13567165726</t>
         </is>
       </c>
       <c r="L22" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-廉村镇段庄村742号</t>
+          <t>河南省-平顶山市-叶县-辛店镇刘庄村989号</t>
         </is>
       </c>
     </row>
@@ -2054,40 +2054,40 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年05月</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>410422201211057651</t>
+          <t>410422201305061108</t>
         </is>
       </c>
       <c r="G23" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>许强</t>
+          <t>于飞</t>
         </is>
       </c>
       <c r="I23" s="14" t="inlineStr">
         <is>
-          <t>13516272046</t>
+          <t>15214737996</t>
         </is>
       </c>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>梁梅</t>
+          <t>宋娜</t>
         </is>
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>18264641708</t>
+          <t>18227354549</t>
         </is>
       </c>
       <c r="L23" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇思城村230号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡蔡庄村570号</t>
         </is>
       </c>
     </row>
@@ -2112,40 +2112,40 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>41042220130731706X</t>
+          <t>410422201210183217</t>
         </is>
       </c>
       <c r="G24" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>李鹏强</t>
+          <t>高俊</t>
         </is>
       </c>
       <c r="I24" s="14" t="inlineStr">
         <is>
-          <t>13932719374</t>
+          <t>15995788568</t>
         </is>
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>谢巧</t>
+          <t>宋欣</t>
         </is>
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>13824190496</t>
+          <t>15844313518</t>
         </is>
       </c>
       <c r="L24" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-田庄乡水郭村78号</t>
+          <t>河南省-平顶山市-叶县-仙台镇老鸦张村197号</t>
         </is>
       </c>
     </row>
@@ -2170,12 +2170,12 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2013年05月</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>410422201301038489</t>
+          <t>410422201305271524</t>
         </is>
       </c>
       <c r="G25" s="13" t="n">
@@ -2183,27 +2183,27 @@
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>罗涛</t>
+          <t>马杰</t>
         </is>
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>13658651850</t>
+          <t>15935240824</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>冯涵怡</t>
+          <t>张静</t>
         </is>
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>18826284987</t>
+          <t>13971094777</t>
         </is>
       </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡李庄村846号</t>
+          <t>河南省-平顶山市-叶县-夏李乡老鸦张村989号</t>
         </is>
       </c>
     </row>
@@ -2228,12 +2228,12 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>410422201301166683</t>
+          <t>410422201302032600</t>
         </is>
       </c>
       <c r="G26" s="13" t="n">
@@ -2241,27 +2241,27 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>林勇晨</t>
+          <t>林涛</t>
         </is>
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>15279965075</t>
+          <t>18799938677</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>孙涵玲</t>
+          <t>罗瑶</t>
         </is>
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>18249480831</t>
+          <t>13691334123</t>
         </is>
       </c>
       <c r="L26" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡李庄村501号</t>
+          <t>河南省-平顶山市-叶县-辛店镇陈庄村77号</t>
         </is>
       </c>
     </row>
@@ -2286,12 +2286,12 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>410422201308202228</t>
+          <t>410422201304294116</t>
         </is>
       </c>
       <c r="G27" s="13" t="n">
@@ -2299,27 +2299,27 @@
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>曹晨</t>
+          <t>张辉鑫</t>
         </is>
       </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
-          <t>13743634957</t>
+          <t>18813493618</t>
         </is>
       </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>傅彤</t>
+          <t>高慧</t>
         </is>
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>19955744431</t>
+          <t>13910249947</t>
         </is>
       </c>
       <c r="L27" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡水郭村324号</t>
+          <t>河南省-平顶山市-叶县-保安镇王庄村706号</t>
         </is>
       </c>
     </row>
@@ -2344,40 +2344,40 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>410422201308203917</t>
+          <t>410422201209146074</t>
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>胡文</t>
+          <t>高强</t>
         </is>
       </c>
       <c r="I28" s="14" t="inlineStr">
         <is>
-          <t>15898941343</t>
+          <t>15890278742</t>
         </is>
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>谢美</t>
+          <t>曾瑶</t>
         </is>
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>19924008427</t>
+          <t>17617565512</t>
         </is>
       </c>
       <c r="L28" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-保安镇小张庄588号</t>
+          <t>河南省-平顶山市-叶县-夏李乡李庄村711号</t>
         </is>
       </c>
     </row>
@@ -2402,40 +2402,40 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>410422201305045617</t>
+          <t>410422201209193452</t>
         </is>
       </c>
       <c r="G29" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>宋刚</t>
+          <t>杨斌涛</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>15871167190</t>
+          <t>18680876038</t>
         </is>
       </c>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>吴慧</t>
+          <t>谢涵</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>15913186999</t>
+          <t>13634824771</t>
         </is>
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡刘庄村390号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇周庄村819号</t>
         </is>
       </c>
     </row>
@@ -2455,45 +2455,45 @@
       </c>
       <c r="D30" s="40" t="inlineStr">
         <is>
-          <t>满族</t>
+          <t>汉</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>410422201301318033</t>
+          <t>410422201210187019</t>
         </is>
       </c>
       <c r="G30" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>曾阳</t>
+          <t>黄博</t>
         </is>
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>13691334123</t>
+          <t>13974846773</t>
         </is>
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>孙曦芳</t>
+          <t>萧曦英</t>
         </is>
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>18779740344</t>
+          <t>17721465840</t>
         </is>
       </c>
       <c r="L30" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡王庄村73号</t>
+          <t>河南省-平顶山市-叶县-常村镇凤岭新村858号</t>
         </is>
       </c>
     </row>
@@ -2518,40 +2518,40 @@
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>410422201301141406</t>
+          <t>410422201212067386</t>
         </is>
       </c>
       <c r="G31" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>曾建华</t>
+          <t>林健峰</t>
         </is>
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>19932421024</t>
+          <t>13657662702</t>
         </is>
       </c>
       <c r="J31" s="14" t="inlineStr">
         <is>
-          <t>彭诺</t>
+          <t>袁婷</t>
         </is>
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>18817464887</t>
+          <t>18818702621</t>
         </is>
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡盆杨村613号</t>
+          <t>河南省-平顶山市-叶县-龚店乡蔡庄村347号</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
-          <t>410422201302136074</t>
+          <t>410422201308122493</t>
         </is>
       </c>
       <c r="G32" s="13" t="n">
@@ -2589,27 +2589,27 @@
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>何强强</t>
+          <t>许健</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>15890278742</t>
+          <t>17680913431</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>曾瑶</t>
+          <t>于娟</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>17617565512</t>
+          <t>13872400504</t>
         </is>
       </c>
       <c r="L32" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡李庄村711号</t>
+          <t>河南省-平顶山市-叶县-夏李乡思城村442号</t>
         </is>
       </c>
     </row>
@@ -2634,40 +2634,40 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F33" s="13" t="inlineStr">
         <is>
-          <t>41042220130806129X</t>
+          <t>410422201212023567</t>
         </is>
       </c>
       <c r="G33" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>傅磊</t>
+          <t>孙勇</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>18245168087</t>
+          <t>18693792374</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
         <is>
-          <t>冯静怡</t>
+          <t>萧玲</t>
         </is>
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>17670348247</t>
+          <t>18848217594</t>
         </is>
       </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-马庄回族乡赵庄村125号</t>
+          <t>河南省-平顶山市-叶县-廉村镇李庄村707号</t>
         </is>
       </c>
     </row>
@@ -2692,40 +2692,40 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>410422201307098642</t>
+          <t>410422201209123052</t>
         </is>
       </c>
       <c r="G34" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>林平</t>
+          <t>唐飞军</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>13586131712</t>
+          <t>17643953394</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>曹燕</t>
+          <t>周娟</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>15867737826</t>
+          <t>13647095214</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡周庄村521号</t>
+          <t>河南省-平顶山市-叶县-夏李乡李庄村180号</t>
         </is>
       </c>
     </row>
@@ -2750,40 +2750,40 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>410422201210068946</t>
+          <t>410422201304287243</t>
         </is>
       </c>
       <c r="G35" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>冯宇</t>
+          <t>吴辉</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>17740449972</t>
+          <t>18685160481</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
         <is>
-          <t>董晴</t>
+          <t>萧怡</t>
         </is>
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>18288675339</t>
+          <t>15896513709</t>
         </is>
       </c>
       <c r="L35" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-田庄乡菜庄村877号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡陈庄村336号</t>
         </is>
       </c>
     </row>
@@ -2808,40 +2808,40 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>410422201209231825</t>
+          <t>410422201304264793</t>
         </is>
       </c>
       <c r="G36" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>程健</t>
+          <t>罗峰磊</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">
         <is>
-          <t>13970289517</t>
+          <t>13647113826</t>
         </is>
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>赵彤</t>
+          <t>萧怡</t>
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr">
         <is>
-          <t>13526217459</t>
+          <t>19969261796</t>
         </is>
       </c>
       <c r="L36" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡段庄村666号</t>
+          <t>河南省-平顶山市-叶县-常村镇孟庄村707号</t>
         </is>
       </c>
     </row>
@@ -2866,12 +2866,12 @@
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>410422201308122493</t>
+          <t>410422201303058922</t>
         </is>
       </c>
       <c r="G37" s="13" t="n">
@@ -2879,27 +2879,27 @@
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>许健</t>
+          <t>谢哲</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>17680913431</t>
+          <t>18306431713</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>于娟</t>
+          <t>彭娜婷</t>
         </is>
       </c>
       <c r="K37" s="14" t="inlineStr">
         <is>
-          <t>13872400504</t>
+          <t>15229318393</t>
         </is>
       </c>
       <c r="L37" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡思城村442号</t>
+          <t>河南省-平顶山市-叶县-任店镇菜庄村337号</t>
         </is>
       </c>
     </row>
@@ -2924,40 +2924,40 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>410422201305303567</t>
+          <t>410422201212318021</t>
         </is>
       </c>
       <c r="G38" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>沈刚勇</t>
+          <t>梁强军</t>
         </is>
       </c>
       <c r="I38" s="14" t="inlineStr">
         <is>
-          <t>18693792374</t>
+          <t>13968117758</t>
         </is>
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>萧玲</t>
+          <t>曾娟</t>
         </is>
       </c>
       <c r="K38" s="14" t="inlineStr">
         <is>
-          <t>18848217594</t>
+          <t>15290847007</t>
         </is>
       </c>
       <c r="L38" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-廉村镇李庄村707号</t>
+          <t>河南省-平顶山市-叶县-任店镇段庄村437号</t>
         </is>
       </c>
     </row>
@@ -2977,45 +2977,45 @@
       </c>
       <c r="D39" s="40" t="inlineStr">
         <is>
-          <t>汉</t>
+          <t>蒙古族</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>41042220130202742X</t>
+          <t>410422201210085251</t>
         </is>
       </c>
       <c r="G39" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>韩豪健</t>
+          <t>杨斌</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>18394406409</t>
+          <t>13724998569</t>
         </is>
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>刘涵</t>
+          <t>邓燕</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>15939533942</t>
+          <t>18711836736</t>
         </is>
       </c>
       <c r="L39" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-廉村镇梅湾村926号</t>
+          <t>河南省-平顶山市-叶县-夏李乡王庄村409号</t>
         </is>
       </c>
     </row>
@@ -3040,40 +3040,40 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr">
         <is>
-          <t>41042220120921792X</t>
+          <t>41042220130311258X</t>
         </is>
       </c>
       <c r="G40" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>董磊</t>
+          <t>程洋勇</t>
         </is>
       </c>
       <c r="I40" s="14" t="inlineStr">
         <is>
-          <t>13914562328</t>
+          <t>13761528098</t>
         </is>
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>谢彤</t>
+          <t>傅婷</t>
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr">
         <is>
-          <t>15824745171</t>
+          <t>18756049451</t>
         </is>
       </c>
       <c r="L40" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-辛店镇菜庄村881号</t>
+          <t>河南省-平顶山市-叶县-水寨乡刘庄村218号</t>
         </is>
       </c>
     </row>
@@ -3098,12 +3098,12 @@
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr">
         <is>
-          <t>410422201303235181</t>
+          <t>410422201302278648</t>
         </is>
       </c>
       <c r="G41" s="13" t="n">
@@ -3111,27 +3111,27 @@
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>傅凯俊</t>
+          <t>傅凯飞</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr">
         <is>
-          <t>13548175496</t>
+          <t>15268998094</t>
         </is>
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>谢娟</t>
+          <t>李美雪</t>
         </is>
       </c>
       <c r="K41" s="14" t="inlineStr">
         <is>
-          <t>17609859317</t>
+          <t>18250229612</t>
         </is>
       </c>
       <c r="L41" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-马庄回族乡凤岭新村665号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡小张庄94号</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
       </c>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>410422201211114711</t>
+          <t>41042220121120639X</t>
         </is>
       </c>
       <c r="G42" s="13" t="n">
@@ -3169,27 +3169,27 @@
       </c>
       <c r="H42" s="14" t="inlineStr">
         <is>
-          <t>张波</t>
+          <t>罗斌</t>
         </is>
       </c>
       <c r="I42" s="14" t="inlineStr">
         <is>
-          <t>13813826758</t>
+          <t>13702290147</t>
         </is>
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>冯慧</t>
+          <t>于涵</t>
         </is>
       </c>
       <c r="K42" s="14" t="inlineStr">
         <is>
-          <t>13879640537</t>
+          <t>18743815614</t>
         </is>
       </c>
       <c r="L42" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡菜庄村876号</t>
+          <t>河南省-平顶山市-叶县-廉村镇孙庄村499号</t>
         </is>
       </c>
     </row>
@@ -3214,40 +3214,40 @@
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
         <is>
-          <t>410422201308183832</t>
+          <t>410422201209294209</t>
         </is>
       </c>
       <c r="G43" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H43" s="14" t="inlineStr">
         <is>
-          <t>许浩飞</t>
+          <t>朱波</t>
         </is>
       </c>
       <c r="I43" s="14" t="inlineStr">
         <is>
-          <t>15117139005</t>
+          <t>13944510762</t>
         </is>
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>林秀英</t>
+          <t>周佳</t>
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr">
         <is>
-          <t>15118393352</t>
+          <t>15288516060</t>
         </is>
       </c>
       <c r="L43" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇周庄村3号</t>
+          <t>河南省-平顶山市-叶县-龚店乡盆杨村883号</t>
         </is>
       </c>
     </row>
@@ -3272,40 +3272,40 @@
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr">
         <is>
-          <t>410422201211067290</t>
+          <t>410422201301278945</t>
         </is>
       </c>
       <c r="G44" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H44" s="14" t="inlineStr">
         <is>
-          <t>何刚强</t>
+          <t>唐强</t>
         </is>
       </c>
       <c r="I44" s="14" t="inlineStr">
         <is>
-          <t>13905395024</t>
+          <t>15097516136</t>
         </is>
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>刘秀英</t>
+          <t>曾悦</t>
         </is>
       </c>
       <c r="K44" s="14" t="inlineStr">
         <is>
-          <t>17711775891</t>
+          <t>18645352181</t>
         </is>
       </c>
       <c r="L44" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡刘庄村227号</t>
+          <t>河南省-平顶山市-叶县-邓李乡刘庄村199号</t>
         </is>
       </c>
     </row>
@@ -3330,12 +3330,12 @@
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年07月</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>410422201308046179</t>
+          <t>410422201307286191</t>
         </is>
       </c>
       <c r="G45" s="13" t="n">
@@ -3343,27 +3343,27 @@
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>罗博</t>
+          <t>吴鹏华</t>
         </is>
       </c>
       <c r="I45" s="14" t="inlineStr">
         <is>
-          <t>13507661771</t>
+          <t>15129212779</t>
         </is>
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>杨琳</t>
+          <t>曾诗</t>
         </is>
       </c>
       <c r="K45" s="14" t="inlineStr">
         <is>
-          <t>13724998569</t>
+          <t>18252717744</t>
         </is>
       </c>
       <c r="L45" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-邓李乡凤岭新村465号</t>
+          <t>河南省-平顶山市-叶县-水寨乡孟庄村361号</t>
         </is>
       </c>
     </row>
@@ -3388,12 +3388,12 @@
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>410422201304091619</t>
+          <t>410422201303087612</t>
         </is>
       </c>
       <c r="G46" s="13" t="n">
@@ -3401,27 +3401,27 @@
       </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
-          <t>黄文</t>
+          <t>马洋</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>15265766156</t>
+          <t>13799867980</t>
         </is>
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>梁玲</t>
+          <t>董诺</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>13971111615</t>
+          <t>18297820715</t>
         </is>
       </c>
       <c r="L46" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇双庄村570号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡盆杨村517号</t>
         </is>
       </c>
     </row>
@@ -3446,12 +3446,12 @@
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>2013年06月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>410422201306156749</t>
+          <t>410422201304137091</t>
         </is>
       </c>
       <c r="G47" s="13" t="n">
@@ -3459,27 +3459,27 @@
       </c>
       <c r="H47" s="14" t="inlineStr">
         <is>
-          <t>宋涛</t>
+          <t>邓平</t>
         </is>
       </c>
       <c r="I47" s="14" t="inlineStr">
         <is>
-          <t>18704945198</t>
+          <t>15966590515</t>
         </is>
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>朱慧</t>
+          <t>赵曦</t>
         </is>
       </c>
       <c r="K47" s="14" t="inlineStr">
         <is>
-          <t>15215851493</t>
+          <t>15949251925</t>
         </is>
       </c>
       <c r="L47" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇李庄村866号</t>
+          <t>河南省-平顶山市-叶县-常村镇段庄村133号</t>
         </is>
       </c>
     </row>
@@ -3504,40 +3504,40 @@
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>410422201307124195</t>
+          <t>410422201211057116</t>
         </is>
       </c>
       <c r="G48" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>傅强</t>
+          <t>邓勇</t>
         </is>
       </c>
       <c r="I48" s="14" t="inlineStr">
         <is>
-          <t>15802445502</t>
+          <t>18785054235</t>
         </is>
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>吴诺</t>
+          <t>曹英秀英</t>
         </is>
       </c>
       <c r="K48" s="14" t="inlineStr">
         <is>
-          <t>13720183667</t>
+          <t>13914188805</t>
         </is>
       </c>
       <c r="L48" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡老鸦张村379号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡周庄村135号</t>
         </is>
       </c>
     </row>
@@ -3562,40 +3562,40 @@
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>2013年06月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>410422201306183094</t>
+          <t>410422201211249934</t>
         </is>
       </c>
       <c r="G49" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
-          <t>杨军军</t>
+          <t>董磊</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>13747679764</t>
+          <t>15279473834</t>
         </is>
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>朱妍瑶</t>
+          <t>程英</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>13849784036</t>
+          <t>18874688623</t>
         </is>
       </c>
       <c r="L49" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡孟庄村8号</t>
+          <t>河南省-平顶山市-叶县-仙台镇周庄村142号</t>
         </is>
       </c>
     </row>
@@ -3620,40 +3620,40 @@
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>2012年12月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr">
         <is>
-          <t>410422201212182176</t>
+          <t>410422201306112492</t>
         </is>
       </c>
       <c r="G50" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>周华涛</t>
+          <t>邓涛平</t>
         </is>
       </c>
       <c r="I50" s="14" t="inlineStr">
         <is>
-          <t>13576226838</t>
+          <t>15878261375</t>
         </is>
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>傅欣敏</t>
+          <t>李璐妍</t>
         </is>
       </c>
       <c r="K50" s="14" t="inlineStr">
         <is>
-          <t>18707159696</t>
+          <t>18336153051</t>
         </is>
       </c>
       <c r="L50" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡李庄村297号</t>
+          <t>河南省-平顶山市-叶县-任店镇杨岭庄村811号</t>
         </is>
       </c>
     </row>
@@ -3678,40 +3678,40 @@
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F51" s="15" t="inlineStr">
         <is>
-          <t>41042220120911844X</t>
+          <t>410422201304306480</t>
         </is>
       </c>
       <c r="G51" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>徐博</t>
+          <t>周豪</t>
         </is>
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>18316136968</t>
+          <t>13510432898</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t>杨悦</t>
+          <t>于霞</t>
         </is>
       </c>
       <c r="K51" s="8" t="inlineStr">
         <is>
-          <t>18235218188</t>
+          <t>15241036971</t>
         </is>
       </c>
       <c r="L51" s="9" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡思城村360号</t>
+          <t>河南省-平顶山市-叶县-保安镇赵庄村612号</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3741,7 @@
       </c>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>410422201211151754</t>
+          <t>410422201211139071</t>
         </is>
       </c>
       <c r="G52" s="13" t="n">
@@ -3749,27 +3749,27 @@
       </c>
       <c r="H52" s="14" t="inlineStr">
         <is>
-          <t>赵超刚</t>
+          <t>于伟</t>
         </is>
       </c>
       <c r="I52" s="14" t="inlineStr">
         <is>
-          <t>13912779979</t>
+          <t>15296218518</t>
         </is>
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>吕琳</t>
+          <t>许妍</t>
         </is>
       </c>
       <c r="K52" s="14" t="inlineStr">
         <is>
-          <t>18227177449</t>
+          <t>17780670654</t>
         </is>
       </c>
       <c r="L52" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇思城村520号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡小张庄366号</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年07月</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>410422201304251868</t>
+          <t>410422201307194650</t>
         </is>
       </c>
       <c r="G53" s="13" t="n">
@@ -3807,27 +3807,27 @@
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>张军</t>
+          <t>曾宇浩</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>15911998679</t>
+          <t>19952772217</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t>傅敏</t>
+          <t>张燕英</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>15159782071</t>
+          <t>13654868740</t>
         </is>
       </c>
       <c r="L53" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇杨岭庄村732号</t>
+          <t>河南省-平顶山市-叶县-仙台镇水郭村293号</t>
         </is>
       </c>
     </row>
@@ -3852,12 +3852,12 @@
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年05月</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>410422201307282535</t>
+          <t>410422201305135454</t>
         </is>
       </c>
       <c r="G54" s="13" t="n">
@@ -3865,27 +3865,27 @@
       </c>
       <c r="H54" s="14" t="inlineStr">
         <is>
-          <t>张鹏</t>
+          <t>曹凯</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>18888925546</t>
+          <t>17741616928</t>
         </is>
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>冯婷</t>
+          <t>马琳琳</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>13651518644</t>
+          <t>15947962757</t>
         </is>
       </c>
       <c r="L54" s="17" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡周庄村895号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇思城村630号</t>
         </is>
       </c>
     </row>
@@ -3910,12 +3910,12 @@
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F55" s="13" t="inlineStr">
         <is>
-          <t>410422201210123312</t>
+          <t>410422201209305075</t>
         </is>
       </c>
       <c r="G55" s="13" t="n">
@@ -3923,27 +3923,27 @@
       </c>
       <c r="H55" s="14" t="inlineStr">
         <is>
-          <t>吴浩</t>
+          <t>唐凯</t>
         </is>
       </c>
       <c r="I55" s="14" t="inlineStr">
         <is>
-          <t>18629148652</t>
+          <t>15002970213</t>
         </is>
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>邓艳</t>
+          <t>谢怡</t>
         </is>
       </c>
       <c r="K55" s="14" t="inlineStr">
         <is>
-          <t>18785054235</t>
+          <t>13692755719</t>
         </is>
       </c>
       <c r="L55" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇赵庄村197号</t>
+          <t>河南省-平顶山市-叶县-辛店镇刘庄村376号</t>
         </is>
       </c>
     </row>
@@ -3968,12 +3968,12 @@
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>410422201211196463</t>
+          <t>41042220120914261X</t>
         </is>
       </c>
       <c r="G56" s="13" t="n">
@@ -3981,27 +3981,27 @@
       </c>
       <c r="H56" s="14" t="inlineStr">
         <is>
-          <t>马杰</t>
+          <t>孙然</t>
         </is>
       </c>
       <c r="I56" s="14" t="inlineStr">
         <is>
-          <t>19980592962</t>
+          <t>19914473947</t>
         </is>
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>徐美</t>
+          <t>胡霞丽</t>
         </is>
       </c>
       <c r="K56" s="14" t="inlineStr">
         <is>
-          <t>15070653794</t>
+          <t>18827155188</t>
         </is>
       </c>
       <c r="L56" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇王庄村240号</t>
+          <t>河南省-平顶山市-叶县-常村镇凤岭新村872号</t>
         </is>
       </c>
     </row>
@@ -4026,40 +4026,40 @@
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>410422201302065608</t>
+          <t>410422201211026295</t>
         </is>
       </c>
       <c r="G57" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H57" s="14" t="inlineStr">
         <is>
-          <t>程建华</t>
+          <t>周鹏</t>
         </is>
       </c>
       <c r="I57" s="14" t="inlineStr">
         <is>
-          <t>18874688623</t>
+          <t>13558957829</t>
         </is>
       </c>
       <c r="J57" s="14" t="inlineStr">
         <is>
-          <t>彭秀英</t>
+          <t>杨丽</t>
         </is>
       </c>
       <c r="K57" s="14" t="inlineStr">
         <is>
-          <t>13675818141</t>
+          <t>17686691251</t>
         </is>
       </c>
       <c r="L57" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇老鸦张村280号</t>
+          <t>河南省-平顶山市-叶县-龚店乡王庄村697号</t>
         </is>
       </c>
     </row>
@@ -4084,40 +4084,40 @@
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
-          <t>410422201211159512</t>
+          <t>410422201306106461</t>
         </is>
       </c>
       <c r="G58" s="14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H58" s="14" t="inlineStr">
         <is>
-          <t>于勇</t>
+          <t>曾刚</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>15275060685</t>
+          <t>13968018242</t>
         </is>
       </c>
       <c r="J58" s="14" t="inlineStr">
         <is>
-          <t>林佳</t>
+          <t>徐琳</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>18330515220</t>
+          <t>15258414384</t>
         </is>
       </c>
       <c r="L58" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇赵庄村713号</t>
+          <t>河南省-平顶山市-叶县-辛店镇凤岭新村630号</t>
         </is>
       </c>
     </row>
@@ -4142,40 +4142,40 @@
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>410422201308286279</t>
+          <t>410422201211185506</t>
         </is>
       </c>
       <c r="G59" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>董伟</t>
+          <t>吕宇</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>13543289861</t>
+          <t>13601094396</t>
         </is>
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>马红</t>
+          <t>吕娜</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>13636971179</t>
+          <t>19944736471</t>
         </is>
       </c>
       <c r="L59" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-邓李乡小张庄648号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡孟庄村162号</t>
         </is>
       </c>
     </row>
@@ -4200,40 +4200,40 @@
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>410422201301029071</t>
+          <t>410422201211138812</t>
         </is>
       </c>
       <c r="G60" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>吴鑫</t>
+          <t>梁浩</t>
         </is>
       </c>
       <c r="I60" s="14" t="inlineStr">
         <is>
-          <t>18339621851</t>
+          <t>13958815371</t>
         </is>
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>邓晴</t>
+          <t>郭诗娟</t>
         </is>
       </c>
       <c r="K60" s="14" t="inlineStr">
         <is>
-          <t>17780670654</t>
+          <t>13646963259</t>
         </is>
       </c>
       <c r="L60" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡小张庄366号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡杨岭庄村195号</t>
         </is>
       </c>
     </row>
@@ -4253,17 +4253,17 @@
       </c>
       <c r="D61" s="40" t="inlineStr">
         <is>
-          <t>汉</t>
+          <t>回族</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2013年05月</t>
         </is>
       </c>
       <c r="F61" s="14" t="inlineStr">
         <is>
-          <t>410422201302244650</t>
+          <t>410422201305142995</t>
         </is>
       </c>
       <c r="G61" s="14" t="n">
@@ -4271,27 +4271,27 @@
       </c>
       <c r="H61" s="14" t="inlineStr">
         <is>
-          <t>赵宇浩</t>
+          <t>罗然俊</t>
         </is>
       </c>
       <c r="I61" s="14" t="inlineStr">
         <is>
-          <t>19952772217</t>
+          <t>17773395004</t>
         </is>
       </c>
       <c r="J61" s="14" t="inlineStr">
         <is>
-          <t>张燕英</t>
+          <t>曹萱芳</t>
         </is>
       </c>
       <c r="K61" s="14" t="inlineStr">
         <is>
-          <t>13654868740</t>
+          <t>13862456506</t>
         </is>
       </c>
       <c r="L61" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇水郭村293号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇孙庄村576号</t>
         </is>
       </c>
     </row>
@@ -4316,12 +4316,12 @@
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
-          <t>410422201308024024</t>
+          <t>410422201304194359</t>
         </is>
       </c>
       <c r="G62" s="14" t="n">
@@ -4329,27 +4329,27 @@
       </c>
       <c r="H62" s="14" t="inlineStr">
         <is>
-          <t>郭涛</t>
+          <t>傅飞</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>18767652775</t>
+          <t>13821655852</t>
         </is>
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>邓玉</t>
+          <t>胡妍</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>18716928451</t>
+          <t>13600257872</t>
         </is>
       </c>
       <c r="L62" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-保安镇杨岭庄村677号</t>
+          <t>河南省-平顶山市-叶县-水寨乡刘庄村144号</t>
         </is>
       </c>
     </row>
@@ -4374,12 +4374,12 @@
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F63" s="14" t="inlineStr">
         <is>
-          <t>410422201304174929</t>
+          <t>410422201302017449</t>
         </is>
       </c>
       <c r="G63" s="14" t="n">
@@ -4387,27 +4387,27 @@
       </c>
       <c r="H63" s="14" t="inlineStr">
         <is>
-          <t>于平</t>
+          <t>宋轩</t>
         </is>
       </c>
       <c r="I63" s="14" t="inlineStr">
         <is>
-          <t>18370596401</t>
+          <t>19979470551</t>
         </is>
       </c>
       <c r="J63" s="14" t="inlineStr">
         <is>
-          <t>唐怡</t>
+          <t>冯雪</t>
         </is>
       </c>
       <c r="K63" s="14" t="inlineStr">
         <is>
-          <t>15002970213</t>
+          <t>13597499309</t>
         </is>
       </c>
       <c r="L63" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇思城村371号</t>
+          <t>河南省-平顶山市-叶县-龚店乡老鸦张村537号</t>
         </is>
       </c>
     </row>
@@ -4432,40 +4432,40 @@
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>410422201209177264</t>
+          <t>410422201303314053</t>
         </is>
       </c>
       <c r="G64" s="14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H64" s="14" t="inlineStr">
         <is>
-          <t>吴晨</t>
+          <t>朱峰</t>
         </is>
       </c>
       <c r="I64" s="14" t="inlineStr">
         <is>
-          <t>18371928565</t>
+          <t>17602838578</t>
         </is>
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>郭红</t>
+          <t>韩琳</t>
         </is>
       </c>
       <c r="K64" s="14" t="inlineStr">
         <is>
-          <t>13527868144</t>
+          <t>18885854973</t>
         </is>
       </c>
       <c r="L64" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡王庄村220号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡蔡庄村572号</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite map: store coords in Student, direct display, CLGeocoder+AMap fallback
</commit_message>
<xml_diff>
--- a/七（4）班学生信息_模拟数据.xlsx
+++ b/七（4）班学生信息_模拟数据.xlsx
@@ -952,40 +952,40 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>410422201210233847</t>
+          <t>410422201303034795</t>
         </is>
       </c>
       <c r="G4" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>韩杰</t>
+          <t>郑华</t>
         </is>
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>18394078161</t>
+          <t>18881618495</t>
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>傅燕</t>
+          <t>沈英</t>
         </is>
       </c>
       <c r="K4" s="14" t="inlineStr">
         <is>
-          <t>18393103413</t>
+          <t>13634131647</t>
         </is>
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-任店镇梅湾村390号</t>
+          <t>河南省-平顶山市-叶县-廉村镇思城村167号</t>
         </is>
       </c>
     </row>
@@ -1010,12 +1010,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>410422201303013712</t>
+          <t>410422201301046976</t>
         </is>
       </c>
       <c r="G5" s="13" t="n">
@@ -1023,27 +1023,27 @@
       </c>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>郭洋</t>
+          <t>萧健辉</t>
         </is>
       </c>
       <c r="I5" s="14" t="inlineStr">
         <is>
-          <t>15083276483</t>
+          <t>18203056413</t>
         </is>
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>梁静敏</t>
+          <t>沈琳涵</t>
         </is>
       </c>
       <c r="K5" s="14" t="inlineStr">
         <is>
-          <t>18264139537</t>
+          <t>18672423884</t>
         </is>
       </c>
       <c r="L5" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-田庄乡王庄村147号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡孙庄村439号</t>
         </is>
       </c>
     </row>
@@ -1063,45 +1063,45 @@
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>汉</t>
+          <t>满族</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>410422201301138381</t>
+          <t>410422201209256122</t>
         </is>
       </c>
       <c r="G6" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>曾阳</t>
+          <t>黄超</t>
         </is>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>18653287101</t>
+          <t>18791669784</t>
         </is>
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>吴巧</t>
+          <t>傅芳</t>
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr">
         <is>
-          <t>18791669784</t>
+          <t>13884514627</t>
         </is>
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-邓李乡小张庄697号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇蔡庄村996号</t>
         </is>
       </c>
     </row>
@@ -1126,40 +1126,40 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>410422201301151593</t>
+          <t>410422201212119939</t>
         </is>
       </c>
       <c r="G7" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7" s="14" t="inlineStr">
         <is>
-          <t>宋涛平</t>
+          <t>谢平</t>
         </is>
       </c>
       <c r="I7" s="14" t="inlineStr">
         <is>
-          <t>18804828148</t>
+          <t>17709570154</t>
         </is>
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>彭英巧</t>
+          <t>林静诺</t>
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr">
         <is>
-          <t>19980957015</t>
+          <t>13717182278</t>
         </is>
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-马庄回族乡凤岭新村246号</t>
+          <t>河南省-平顶山市-叶县-辛店镇蔡庄村541号</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>410422201307084381</t>
+          <t>410422201302078409</t>
         </is>
       </c>
       <c r="G8" s="13" t="n">
@@ -1197,27 +1197,27 @@
       </c>
       <c r="H8" s="14" t="inlineStr">
         <is>
-          <t>朱哲</t>
+          <t>谢晨</t>
         </is>
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
-          <t>15146578713</t>
+          <t>18813315098</t>
         </is>
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>高丽</t>
+          <t>高萍静</t>
         </is>
       </c>
       <c r="K8" s="14" t="inlineStr">
         <is>
-          <t>19939301031</t>
+          <t>15210518347</t>
         </is>
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-马庄回族乡孟庄村881号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡陈庄村136号</t>
         </is>
       </c>
     </row>
@@ -1242,12 +1242,12 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>2012年12月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>410422201212199951</t>
+          <t>410422201210201151</t>
         </is>
       </c>
       <c r="G9" s="13" t="n">
@@ -1255,27 +1255,27 @@
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>周豪豪</t>
+          <t>于浩</t>
         </is>
       </c>
       <c r="I9" s="14" t="inlineStr">
         <is>
-          <t>18731165667</t>
+          <t>18801065133</t>
         </is>
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>刘娟婷</t>
+          <t>胡晴</t>
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr">
         <is>
-          <t>13833387262</t>
+          <t>18724731781</t>
         </is>
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇王庄村256号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇陈庄村857号</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1300,12 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>2013年06月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>410422201306098538</t>
+          <t>410422201304212229</t>
         </is>
       </c>
       <c r="G10" s="13" t="n">
@@ -1313,27 +1313,27 @@
       </c>
       <c r="H10" s="14" t="inlineStr">
         <is>
-          <t>刘哲</t>
+          <t>于然鑫</t>
         </is>
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
-          <t>13732677360</t>
+          <t>15109805009</t>
         </is>
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>徐佳佳</t>
+          <t>程妍</t>
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr">
         <is>
-          <t>15874687234</t>
+          <t>17720812191</t>
         </is>
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡孟庄村594号</t>
+          <t>河南省-平顶山市-叶县-廉村镇菜庄村414号</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>41042220130627787X</t>
+          <t>410422201306263912</t>
         </is>
       </c>
       <c r="G11" s="13" t="n">
@@ -1371,27 +1371,27 @@
       </c>
       <c r="H11" s="14" t="inlineStr">
         <is>
-          <t>袁睿轩</t>
+          <t>邓斌</t>
         </is>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
-          <t>13721913619</t>
+          <t>15153462475</t>
         </is>
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>林敏</t>
+          <t>陈芳</t>
         </is>
       </c>
       <c r="K11" s="14" t="inlineStr">
         <is>
-          <t>18799854353</t>
+          <t>13818384251</t>
         </is>
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇段庄村135号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡菜庄村379号</t>
         </is>
       </c>
     </row>
@@ -1416,40 +1416,40 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>410422201209053784</t>
+          <t>410422201308018892</t>
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H12" s="14" t="inlineStr">
         <is>
-          <t>吕杰文</t>
+          <t>王波</t>
         </is>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>17742513542</t>
+          <t>13824118244</t>
         </is>
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>董晴</t>
+          <t>彭梅</t>
         </is>
       </c>
       <c r="K12" s="14" t="inlineStr">
         <is>
-          <t>17708412411</t>
+          <t>15148740164</t>
         </is>
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡陈庄村160号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇小张庄342号</t>
         </is>
       </c>
     </row>
@@ -1474,12 +1474,12 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>2012年12月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>410422201212145402</t>
+          <t>410422201209052835</t>
         </is>
       </c>
       <c r="G13" s="13" t="n">
@@ -1487,27 +1487,27 @@
       </c>
       <c r="H13" s="14" t="inlineStr">
         <is>
-          <t>何轩</t>
+          <t>陈超</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
         <is>
-          <t>13616400524</t>
+          <t>18398262045</t>
         </is>
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>徐诗</t>
+          <t>张欣红</t>
         </is>
       </c>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>18780112805</t>
+          <t>13858692322</t>
         </is>
       </c>
       <c r="L13" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡陈庄村152号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡李庄村26号</t>
         </is>
       </c>
     </row>
@@ -1532,40 +1532,40 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>410422201303034123</t>
+          <t>410422201212266903</t>
         </is>
       </c>
       <c r="G14" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H14" s="14" t="inlineStr">
         <is>
-          <t>林杰</t>
+          <t>李建华</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>19969232260</t>
+          <t>15814586850</t>
         </is>
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>孙婷</t>
+          <t>黄玲玲</t>
         </is>
       </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>18734216073</t>
+          <t>13619655698</t>
         </is>
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡王庄村359号</t>
+          <t>河南省-平顶山市-叶县-保安镇段庄村922号</t>
         </is>
       </c>
     </row>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>410422201303245460</t>
+          <t>410422201306033933</t>
         </is>
       </c>
       <c r="G15" s="13" t="n">
@@ -1603,27 +1603,27 @@
       </c>
       <c r="H15" s="14" t="inlineStr">
         <is>
-          <t>郭洋</t>
+          <t>胡凯</t>
         </is>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
-          <t>15858685014</t>
+          <t>18295148465</t>
         </is>
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>孙玲瑶</t>
+          <t>唐燕</t>
         </is>
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>18356981693</t>
+          <t>15166299468</t>
         </is>
       </c>
       <c r="L15" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇孟庄村726号</t>
+          <t>河南省-平顶山市-叶县-任店镇小张庄312号</t>
         </is>
       </c>
     </row>
@@ -1648,12 +1648,12 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>410422201308183933</t>
+          <t>41042220130415251X</t>
         </is>
       </c>
       <c r="G16" s="13" t="n">
@@ -1661,27 +1661,27 @@
       </c>
       <c r="H16" s="14" t="inlineStr">
         <is>
-          <t>胡凯</t>
+          <t>朱轩</t>
         </is>
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
-          <t>18295148465</t>
+          <t>15014895134</t>
         </is>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>唐燕</t>
+          <t>高英敏</t>
         </is>
       </c>
       <c r="K16" s="14" t="inlineStr">
         <is>
-          <t>15166299468</t>
+          <t>15279176936</t>
         </is>
       </c>
       <c r="L16" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-任店镇小张庄312号</t>
+          <t>河南省-平顶山市-叶县-龚店乡段庄村250号</t>
         </is>
       </c>
     </row>
@@ -1706,12 +1706,12 @@
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>410422201308027449</t>
+          <t>410422201304068968</t>
         </is>
       </c>
       <c r="G17" s="13" t="n">
@@ -1719,27 +1719,27 @@
       </c>
       <c r="H17" s="14" t="inlineStr">
         <is>
-          <t>萧晨</t>
+          <t>孙睿</t>
         </is>
       </c>
       <c r="I17" s="14" t="inlineStr">
         <is>
-          <t>15187214895</t>
+          <t>19931727889</t>
         </is>
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>杨红</t>
+          <t>梁诗</t>
         </is>
       </c>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>15232003791</t>
+          <t>17768727743</t>
         </is>
       </c>
       <c r="L17" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡李庄村908号</t>
+          <t>河南省-平顶山市-叶县-任店镇蔡庄村785号</t>
         </is>
       </c>
     </row>
@@ -1764,12 +1764,12 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>410422201305122627</t>
+          <t>410422201301189556</t>
         </is>
       </c>
       <c r="G18" s="13" t="n">
@@ -1777,27 +1777,27 @@
       </c>
       <c r="H18" s="14" t="inlineStr">
         <is>
-          <t>林超</t>
+          <t>梁哲超</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>13516328708</t>
+          <t>15262316658</t>
         </is>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>林霞</t>
+          <t>萧璐璐</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>18888957986</t>
+          <t>18690967054</t>
         </is>
       </c>
       <c r="L18" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-任店镇陈庄村457号</t>
+          <t>河南省-平顶山市-叶县-仙台镇段庄村874号</t>
         </is>
       </c>
     </row>
@@ -1822,12 +1822,12 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年05月</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>410422201307245306</t>
+          <t>410422201305084456</t>
         </is>
       </c>
       <c r="G19" s="13" t="n">
@@ -1835,27 +1835,27 @@
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>邓然</t>
+          <t>郭阳</t>
         </is>
       </c>
       <c r="I19" s="14" t="inlineStr">
         <is>
-          <t>15871434558</t>
+          <t>18656272980</t>
         </is>
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>杨秀英佳</t>
+          <t>唐诺</t>
         </is>
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>13931665876</t>
+          <t>13762720465</t>
         </is>
       </c>
       <c r="L19" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇水郭村853号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡王庄村335号</t>
         </is>
       </c>
     </row>
@@ -1880,12 +1880,12 @@
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>2013年06月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>410422201306074345</t>
+          <t>410422201304291264</t>
         </is>
       </c>
       <c r="G20" s="13" t="n">
@@ -1893,27 +1893,27 @@
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
-          <t>彭辉</t>
+          <t>许军</t>
         </is>
       </c>
       <c r="I20" s="14" t="inlineStr">
         <is>
-          <t>15867065627</t>
+          <t>18331003309</t>
         </is>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>周晴悦</t>
+          <t>吴红霞</t>
         </is>
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>13516272046</t>
+          <t>15174529912</t>
         </is>
       </c>
       <c r="L20" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡水郭村466号</t>
+          <t>河南省-平顶山市-叶县-常村镇梅湾村593号</t>
         </is>
       </c>
     </row>
@@ -1938,40 +1938,40 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>410422201302274199</t>
+          <t>410422201212119278</t>
         </is>
       </c>
       <c r="G21" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
-          <t>陈磊</t>
+          <t>曾鹏波</t>
         </is>
       </c>
       <c r="I21" s="14" t="inlineStr">
         <is>
-          <t>15230923271</t>
+          <t>13890586518</t>
         </is>
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>沈梅</t>
+          <t>宋芳</t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>15852991241</t>
+          <t>17616572628</t>
         </is>
       </c>
       <c r="L21" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡小张庄952号</t>
+          <t>河南省-平顶山市-叶县-廉村镇蔡庄村631号</t>
         </is>
       </c>
     </row>
@@ -1996,12 +1996,12 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>410422201303237664</t>
+          <t>410422201302203494</t>
         </is>
       </c>
       <c r="G22" s="13" t="n">
@@ -2009,27 +2009,27 @@
       </c>
       <c r="H22" s="14" t="inlineStr">
         <is>
-          <t>胡洋</t>
+          <t>曹斌文</t>
         </is>
       </c>
       <c r="I22" s="14" t="inlineStr">
         <is>
-          <t>15214919058</t>
+          <t>18345494808</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>于怡婷</t>
+          <t>胡艳璐</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>13567165726</t>
+          <t>17683777014</t>
         </is>
       </c>
       <c r="L22" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-辛店镇刘庄村989号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡段庄村709号</t>
         </is>
       </c>
     </row>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>410422201305061108</t>
+          <t>410422201306096462</t>
         </is>
       </c>
       <c r="G23" s="13" t="n">
@@ -2067,27 +2067,27 @@
       </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
-          <t>于飞</t>
+          <t>郑博华</t>
         </is>
       </c>
       <c r="I23" s="14" t="inlineStr">
         <is>
-          <t>15214737996</t>
+          <t>15213518233</t>
         </is>
       </c>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>宋娜</t>
+          <t>程玉</t>
         </is>
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>18227354549</t>
+          <t>17794134352</t>
         </is>
       </c>
       <c r="L23" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡蔡庄村570号</t>
+          <t>河南省-平顶山市-叶县-常村镇小张庄726号</t>
         </is>
       </c>
     </row>
@@ -2112,12 +2112,12 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>410422201210183217</t>
+          <t>410422201211045269</t>
         </is>
       </c>
       <c r="G24" s="13" t="n">
@@ -2125,27 +2125,27 @@
       </c>
       <c r="H24" s="14" t="inlineStr">
         <is>
-          <t>高俊</t>
+          <t>曹杰</t>
         </is>
       </c>
       <c r="I24" s="14" t="inlineStr">
         <is>
-          <t>15995788568</t>
+          <t>15977752047</t>
         </is>
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>宋欣</t>
+          <t>黄丽</t>
         </is>
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>15844313518</t>
+          <t>13790229413</t>
         </is>
       </c>
       <c r="L24" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇老鸦张村197号</t>
+          <t>河南省-平顶山市-叶县-保安镇陈庄村783号</t>
         </is>
       </c>
     </row>
@@ -2170,12 +2170,12 @@
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>410422201305271524</t>
+          <t>410422201304158033</t>
         </is>
       </c>
       <c r="G25" s="13" t="n">
@@ -2183,27 +2183,27 @@
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>马杰</t>
+          <t>曾阳</t>
         </is>
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>15935240824</t>
+          <t>13691334123</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>张静</t>
+          <t>孙曦芳</t>
         </is>
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>13971094777</t>
+          <t>18779740344</t>
         </is>
       </c>
       <c r="L25" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡老鸦张村989号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡王庄村73号</t>
         </is>
       </c>
     </row>
@@ -2228,12 +2228,12 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>410422201302032600</t>
+          <t>41042220130126631X</t>
         </is>
       </c>
       <c r="G26" s="13" t="n">
@@ -2241,27 +2241,27 @@
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>林涛</t>
+          <t>黄博</t>
         </is>
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>18799938677</t>
+          <t>18648877190</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>罗瑶</t>
+          <t>于琳</t>
         </is>
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>13691334123</t>
+          <t>13513990490</t>
         </is>
       </c>
       <c r="L26" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-辛店镇陈庄村77号</t>
+          <t>河南省-平顶山市-叶县-仙台镇老鸦张村482号</t>
         </is>
       </c>
     </row>
@@ -2286,40 +2286,40 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>410422201304294116</t>
+          <t>410422201210177377</t>
         </is>
       </c>
       <c r="G27" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H27" s="14" t="inlineStr">
         <is>
-          <t>张辉鑫</t>
+          <t>郑峰</t>
         </is>
       </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
-          <t>18813493618</t>
+          <t>13825674680</t>
         </is>
       </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>高慧</t>
+          <t>萧艳</t>
         </is>
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>13910249947</t>
+          <t>18216808760</t>
         </is>
       </c>
       <c r="L27" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-保安镇王庄村706号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡刘庄村371号</t>
         </is>
       </c>
     </row>
@@ -2344,40 +2344,40 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>410422201209146074</t>
+          <t>410422201301264923</t>
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H28" s="14" t="inlineStr">
         <is>
-          <t>高强</t>
+          <t>曹涛鹏</t>
         </is>
       </c>
       <c r="I28" s="14" t="inlineStr">
         <is>
-          <t>15890278742</t>
+          <t>15048086131</t>
         </is>
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>曾瑶</t>
+          <t>萧霞</t>
         </is>
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>17617565512</t>
+          <t>13974846773</t>
         </is>
       </c>
       <c r="L28" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡李庄村711号</t>
+          <t>河南省-平顶山市-叶县-龚店乡陈庄村149号</t>
         </is>
       </c>
     </row>
@@ -2402,40 +2402,40 @@
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>410422201209193452</t>
+          <t>410422201308049901</t>
         </is>
       </c>
       <c r="G29" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H29" s="14" t="inlineStr">
         <is>
-          <t>杨斌涛</t>
+          <t>吴晨</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>18680876038</t>
+          <t>18358867533</t>
         </is>
       </c>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>谢涵</t>
+          <t>沈佳璐</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>13634824771</t>
+          <t>13657662702</t>
         </is>
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇周庄村819号</t>
+          <t>河南省-平顶山市-叶县-邓李乡孙庄村340号</t>
         </is>
       </c>
     </row>
@@ -2460,40 +2460,40 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>2012年10月</t>
+          <t>2013年07月</t>
         </is>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>410422201210187019</t>
+          <t>410422201307302493</t>
         </is>
       </c>
       <c r="G30" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H30" s="14" t="inlineStr">
         <is>
-          <t>黄博</t>
+          <t>宋哲</t>
         </is>
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>13974846773</t>
+          <t>18278091343</t>
         </is>
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>萧曦英</t>
+          <t>杨瑶</t>
         </is>
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>17721465840</t>
+          <t>13872400504</t>
         </is>
       </c>
       <c r="L30" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇凤岭新村858号</t>
+          <t>河南省-平顶山市-叶县-夏李乡思城村442号</t>
         </is>
       </c>
     </row>
@@ -2518,12 +2518,12 @@
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>2012年12月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>410422201212067386</t>
+          <t>410422201210114679</t>
         </is>
       </c>
       <c r="G31" s="13" t="n">
@@ -2531,27 +2531,27 @@
       </c>
       <c r="H31" s="14" t="inlineStr">
         <is>
-          <t>林健峰</t>
+          <t>韩鹏</t>
         </is>
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>13657662702</t>
+          <t>13937474074</t>
         </is>
       </c>
       <c r="J31" s="14" t="inlineStr">
         <is>
-          <t>袁婷</t>
+          <t>许巧欣</t>
         </is>
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>18818702621</t>
+          <t>15964743671</t>
         </is>
       </c>
       <c r="L31" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡蔡庄村347号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡段庄村586号</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>2013年08月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
-          <t>410422201308122493</t>
+          <t>410422201303223052</t>
         </is>
       </c>
       <c r="G32" s="13" t="n">
@@ -2589,27 +2589,27 @@
       </c>
       <c r="H32" s="14" t="inlineStr">
         <is>
-          <t>许健</t>
+          <t>王军</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>17680913431</t>
+          <t>17643953394</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>于娟</t>
+          <t>周娟</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>13872400504</t>
+          <t>13647095214</t>
         </is>
       </c>
       <c r="L32" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡思城村442号</t>
+          <t>河南省-平顶山市-叶县-夏李乡李庄村180号</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="D33" s="40" t="inlineStr">
         <is>
-          <t>汉</t>
+          <t>满族</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="F33" s="13" t="inlineStr">
         <is>
-          <t>410422201212023567</t>
+          <t>410422201212255181</t>
         </is>
       </c>
       <c r="G33" s="13" t="n">
@@ -2647,27 +2647,27 @@
       </c>
       <c r="H33" s="14" t="inlineStr">
         <is>
-          <t>孙勇</t>
+          <t>唐凯俊</t>
         </is>
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>18693792374</t>
+          <t>13548175496</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
         <is>
-          <t>萧玲</t>
+          <t>谢娟</t>
         </is>
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>18848217594</t>
+          <t>17609859317</t>
         </is>
       </c>
       <c r="L33" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-廉村镇李庄村707号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡凤岭新村665号</t>
         </is>
       </c>
     </row>
@@ -2692,12 +2692,12 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F34" s="15" t="inlineStr">
         <is>
-          <t>410422201209123052</t>
+          <t>410422201210202941</t>
         </is>
       </c>
       <c r="G34" s="13" t="n">
@@ -2705,27 +2705,27 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>唐飞军</t>
+          <t>许明</t>
         </is>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
-          <t>17643953394</t>
+          <t>18386926179</t>
         </is>
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>周娟</t>
+          <t>冯玉怡</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>13647095214</t>
+          <t>15177351585</t>
         </is>
       </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡李庄村180号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇段庄村283号</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>410422201304287243</t>
+          <t>410422201306115318</t>
         </is>
       </c>
       <c r="G35" s="13" t="n">
@@ -2763,27 +2763,27 @@
       </c>
       <c r="H35" s="14" t="inlineStr">
         <is>
-          <t>吴辉</t>
+          <t>曾文</t>
         </is>
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>18685160481</t>
+          <t>15252904228</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
         <is>
-          <t>萧怡</t>
+          <t>何美娜</t>
         </is>
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>15896513709</t>
+          <t>13905395024</t>
         </is>
       </c>
       <c r="L35" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-马庄回族乡陈庄村336号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇双庄村760号</t>
         </is>
       </c>
     </row>
@@ -2808,40 +2808,40 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2012年10月</t>
         </is>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>410422201304264793</t>
+          <t>410422201210268295</t>
         </is>
       </c>
       <c r="G36" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H36" s="14" t="inlineStr">
         <is>
-          <t>罗峰磊</t>
+          <t>袁辉</t>
         </is>
       </c>
       <c r="I36" s="14" t="inlineStr">
         <is>
-          <t>13647113826</t>
+          <t>13684700766</t>
         </is>
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>萧怡</t>
+          <t>赵涵</t>
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr">
         <is>
-          <t>19969261796</t>
+          <t>18811592124</t>
         </is>
       </c>
       <c r="L36" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇孟庄村707号</t>
+          <t>河南省-平顶山市-叶县-水寨乡孙庄村562号</t>
         </is>
       </c>
     </row>
@@ -2866,12 +2866,12 @@
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F37" s="13" t="inlineStr">
         <is>
-          <t>410422201303058922</t>
+          <t>410422201304091619</t>
         </is>
       </c>
       <c r="G37" s="13" t="n">
@@ -2879,27 +2879,27 @@
       </c>
       <c r="H37" s="14" t="inlineStr">
         <is>
-          <t>谢哲</t>
+          <t>黄文</t>
         </is>
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>18306431713</t>
+          <t>15265766156</t>
         </is>
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>彭娜婷</t>
+          <t>梁玲</t>
         </is>
       </c>
       <c r="K37" s="14" t="inlineStr">
         <is>
-          <t>15229318393</t>
+          <t>13971111615</t>
         </is>
       </c>
       <c r="L37" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-任店镇菜庄村337号</t>
+          <t>河南省-平顶山市-叶县-仙台镇双庄村570号</t>
         </is>
       </c>
     </row>
@@ -2924,40 +2924,40 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>2012年12月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F38" s="13" t="inlineStr">
         <is>
-          <t>410422201212318021</t>
+          <t>41042220130803245X</t>
         </is>
       </c>
       <c r="G38" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H38" s="14" t="inlineStr">
         <is>
-          <t>梁强军</t>
+          <t>高杰</t>
         </is>
       </c>
       <c r="I38" s="14" t="inlineStr">
         <is>
-          <t>13968117758</t>
+          <t>19951493689</t>
         </is>
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>曾娟</t>
+          <t>吕曦玉</t>
         </is>
       </c>
       <c r="K38" s="14" t="inlineStr">
         <is>
-          <t>15290847007</t>
+          <t>13524455022</t>
         </is>
       </c>
       <c r="L38" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-任店镇段庄村437号</t>
+          <t>河南省-平顶山市-叶县-水寨乡段庄村72号</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="D39" s="40" t="inlineStr">
         <is>
-          <t>蒙古族</t>
+          <t>回族</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="F39" s="13" t="inlineStr">
         <is>
-          <t>410422201210085251</t>
+          <t>410422201210143094</t>
         </is>
       </c>
       <c r="G39" s="13" t="n">
@@ -2995,27 +2995,27 @@
       </c>
       <c r="H39" s="14" t="inlineStr">
         <is>
-          <t>杨斌</t>
+          <t>刘超军</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>13724998569</t>
+          <t>13747679764</t>
         </is>
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>邓燕</t>
+          <t>朱妍瑶</t>
         </is>
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>18711836736</t>
+          <t>13849784036</t>
         </is>
       </c>
       <c r="L39" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-夏李乡王庄村409号</t>
+          <t>河南省-平顶山市-叶县-水寨乡孟庄村8号</t>
         </is>
       </c>
     </row>
@@ -3040,12 +3040,12 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年08月</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr">
         <is>
-          <t>41042220130311258X</t>
+          <t>410422201308095108</t>
         </is>
       </c>
       <c r="G40" s="13" t="n">
@@ -3053,27 +3053,27 @@
       </c>
       <c r="H40" s="14" t="inlineStr">
         <is>
-          <t>程洋勇</t>
+          <t>郑洋</t>
         </is>
       </c>
       <c r="I40" s="14" t="inlineStr">
         <is>
-          <t>13761528098</t>
+          <t>13660715969</t>
         </is>
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>傅婷</t>
+          <t>唐璐悦</t>
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr">
         <is>
-          <t>18756049451</t>
+          <t>13552975161</t>
         </is>
       </c>
       <c r="L40" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡刘庄村218号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡李庄村604号</t>
         </is>
       </c>
     </row>
@@ -3098,40 +3098,40 @@
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F41" s="13" t="inlineStr">
         <is>
-          <t>410422201302278648</t>
+          <t>410422201211265501</t>
         </is>
       </c>
       <c r="G41" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H41" s="14" t="inlineStr">
         <is>
-          <t>傅凯飞</t>
+          <t>袁涛</t>
         </is>
       </c>
       <c r="I41" s="14" t="inlineStr">
         <is>
-          <t>15268998094</t>
+          <t>15155231243</t>
         </is>
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>李美雪</t>
+          <t>孙慧</t>
         </is>
       </c>
       <c r="K41" s="14" t="inlineStr">
         <is>
-          <t>18250229612</t>
+          <t>13727799799</t>
         </is>
       </c>
       <c r="L41" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡小张庄94号</t>
+          <t>河南省-平顶山市-叶县-夏李乡杨岭庄村155号</t>
         </is>
       </c>
     </row>
@@ -3156,40 +3156,40 @@
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F42" s="13" t="inlineStr">
         <is>
-          <t>41042220121120639X</t>
+          <t>410422201302289305</t>
         </is>
       </c>
       <c r="G42" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H42" s="14" t="inlineStr">
         <is>
-          <t>罗斌</t>
+          <t>陈波</t>
         </is>
       </c>
       <c r="I42" s="14" t="inlineStr">
         <is>
-          <t>13702290147</t>
+          <t>13605411998</t>
         </is>
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>于涵</t>
+          <t>韩琪</t>
         </is>
       </c>
       <c r="K42" s="14" t="inlineStr">
         <is>
-          <t>18743815614</t>
+          <t>13679359782</t>
         </is>
       </c>
       <c r="L42" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-廉村镇孙庄村499号</t>
+          <t>河南省-平顶山市-叶县-叶邑镇王庄村106号</t>
         </is>
       </c>
     </row>
@@ -3214,40 +3214,40 @@
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
         <is>
-          <t>410422201209294209</t>
+          <t>41042220130318230X</t>
         </is>
       </c>
       <c r="G43" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H43" s="14" t="inlineStr">
         <is>
-          <t>朱波</t>
+          <t>宋军</t>
         </is>
       </c>
       <c r="I43" s="14" t="inlineStr">
         <is>
-          <t>13944510762</t>
+          <t>18215186449</t>
         </is>
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>周佳</t>
+          <t>吴婷慧</t>
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr">
         <is>
-          <t>15288516060</t>
+          <t>18346291486</t>
         </is>
       </c>
       <c r="L43" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡盆杨村883号</t>
+          <t>河南省-平顶山市-叶县-廉村镇杨岭庄村833号</t>
         </is>
       </c>
     </row>
@@ -3272,40 +3272,40 @@
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>2013年01月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F44" s="13" t="inlineStr">
         <is>
-          <t>410422201301278945</t>
+          <t>410422201212084167</t>
         </is>
       </c>
       <c r="G44" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H44" s="14" t="inlineStr">
         <is>
-          <t>唐强</t>
+          <t>周超杰</t>
         </is>
       </c>
       <c r="I44" s="14" t="inlineStr">
         <is>
-          <t>15097516136</t>
+          <t>17788059296</t>
         </is>
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>曾悦</t>
+          <t>吴巧巧</t>
         </is>
       </c>
       <c r="K44" s="14" t="inlineStr">
         <is>
-          <t>18645352181</t>
+          <t>18806537947</t>
         </is>
       </c>
       <c r="L44" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-邓李乡刘庄村199号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡陈庄村245号</t>
         </is>
       </c>
     </row>
@@ -3325,45 +3325,45 @@
       </c>
       <c r="D45" s="40" t="inlineStr">
         <is>
-          <t>汉</t>
+          <t>满族</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F45" s="13" t="inlineStr">
         <is>
-          <t>410422201307286191</t>
+          <t>410422201211101835</t>
         </is>
       </c>
       <c r="G45" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H45" s="14" t="inlineStr">
         <is>
-          <t>吴鹏华</t>
+          <t>何军</t>
         </is>
       </c>
       <c r="I45" s="14" t="inlineStr">
         <is>
-          <t>15129212779</t>
+          <t>18381814124</t>
         </is>
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>曾诗</t>
+          <t>董妍瑶</t>
         </is>
       </c>
       <c r="K45" s="14" t="inlineStr">
         <is>
-          <t>18252717744</t>
+          <t>13737506068</t>
         </is>
       </c>
       <c r="L45" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡孟庄村361号</t>
+          <t>河南省-平顶山市-叶县-夏李乡菜庄村396号</t>
         </is>
       </c>
     </row>
@@ -3388,40 +3388,40 @@
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F46" s="13" t="inlineStr">
         <is>
-          <t>410422201303087612</t>
+          <t>410422201211141641</t>
         </is>
       </c>
       <c r="G46" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H46" s="14" t="inlineStr">
         <is>
-          <t>马洋</t>
+          <t>张鑫</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>13799867980</t>
+          <t>17627790104</t>
         </is>
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>董诺</t>
+          <t>朱慧</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>18297820715</t>
+          <t>17761434103</t>
         </is>
       </c>
       <c r="L46" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡盆杨村517号</t>
+          <t>河南省-平顶山市-叶县-田庄乡周庄村469号</t>
         </is>
       </c>
     </row>
@@ -3446,40 +3446,40 @@
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F47" s="13" t="inlineStr">
         <is>
-          <t>410422201304137091</t>
+          <t>410422201212056595</t>
         </is>
       </c>
       <c r="G47" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H47" s="14" t="inlineStr">
         <is>
-          <t>邓平</t>
+          <t>杨睿</t>
         </is>
       </c>
       <c r="I47" s="14" t="inlineStr">
         <is>
-          <t>15966590515</t>
+          <t>13788888067</t>
         </is>
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>赵曦</t>
+          <t>张佳</t>
         </is>
       </c>
       <c r="K47" s="14" t="inlineStr">
         <is>
-          <t>15949251925</t>
+          <t>15805153195</t>
         </is>
       </c>
       <c r="L47" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇段庄村133号</t>
+          <t>河南省-平顶山市-叶县-辛店镇孟庄村361号</t>
         </is>
       </c>
     </row>
@@ -3504,40 +3504,40 @@
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>410422201211057116</t>
+          <t>410422201302065409</t>
         </is>
       </c>
       <c r="G48" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H48" s="14" t="inlineStr">
         <is>
-          <t>邓勇</t>
+          <t>唐哲</t>
         </is>
       </c>
       <c r="I48" s="14" t="inlineStr">
         <is>
-          <t>18785054235</t>
+          <t>13634505415</t>
         </is>
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>曹英秀英</t>
+          <t>于悦</t>
         </is>
       </c>
       <c r="K48" s="14" t="inlineStr">
         <is>
-          <t>13914188805</t>
+          <t>18652775841</t>
         </is>
       </c>
       <c r="L48" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-马庄回族乡周庄村135号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡李庄村81号</t>
         </is>
       </c>
     </row>
@@ -3562,40 +3562,40 @@
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年04月</t>
         </is>
       </c>
       <c r="F49" s="13" t="inlineStr">
         <is>
-          <t>410422201211249934</t>
+          <t>410422201304172408</t>
         </is>
       </c>
       <c r="G49" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H49" s="14" t="inlineStr">
         <is>
-          <t>董磊</t>
+          <t>郑阳军</t>
         </is>
       </c>
       <c r="I49" s="5" t="inlineStr">
         <is>
-          <t>15279473834</t>
+          <t>13765820297</t>
         </is>
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>程英</t>
+          <t>张秀英怡</t>
         </is>
       </c>
       <c r="K49" s="5" t="inlineStr">
         <is>
-          <t>18874688623</t>
+          <t>18369092755</t>
         </is>
       </c>
       <c r="L49" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇周庄村142号</t>
+          <t>河南省-平顶山市-叶县-龚店乡盆杨村588号</t>
         </is>
       </c>
     </row>
@@ -3620,40 +3620,40 @@
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>2013年06月</t>
+          <t>2012年12月</t>
         </is>
       </c>
       <c r="F50" s="13" t="inlineStr">
         <is>
-          <t>410422201306112492</t>
+          <t>41042220121205261X</t>
         </is>
       </c>
       <c r="G50" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H50" s="14" t="inlineStr">
         <is>
-          <t>邓涛平</t>
+          <t>邓健</t>
         </is>
       </c>
       <c r="I50" s="14" t="inlineStr">
         <is>
-          <t>15878261375</t>
+          <t>13844739473</t>
         </is>
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>李璐妍</t>
+          <t>黄秀英</t>
         </is>
       </c>
       <c r="K50" s="14" t="inlineStr">
         <is>
-          <t>18336153051</t>
+          <t>18827155188</t>
         </is>
       </c>
       <c r="L50" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-任店镇杨岭庄村811号</t>
+          <t>河南省-平顶山市-叶县-常村镇凤岭新村872号</t>
         </is>
       </c>
     </row>
@@ -3678,40 +3678,40 @@
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F51" s="15" t="inlineStr">
         <is>
-          <t>410422201304306480</t>
+          <t>410422201211119488</t>
         </is>
       </c>
       <c r="G51" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H51" s="8" t="inlineStr">
         <is>
-          <t>周豪</t>
+          <t>曹强</t>
         </is>
       </c>
       <c r="I51" s="8" t="inlineStr">
         <is>
-          <t>13510432898</t>
+          <t>18378291146</t>
         </is>
       </c>
       <c r="J51" s="8" t="inlineStr">
         <is>
-          <t>于霞</t>
+          <t>程彤</t>
         </is>
       </c>
       <c r="K51" s="8" t="inlineStr">
         <is>
-          <t>15241036971</t>
+          <t>18791251778</t>
         </is>
       </c>
       <c r="L51" s="9" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-保安镇赵庄村612号</t>
+          <t>河南省-平顶山市-叶县-夏李乡双庄村900号</t>
         </is>
       </c>
     </row>
@@ -3736,12 +3736,12 @@
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2012年09月</t>
         </is>
       </c>
       <c r="F52" s="13" t="inlineStr">
         <is>
-          <t>410422201211139071</t>
+          <t>410422201209299629</t>
         </is>
       </c>
       <c r="G52" s="13" t="n">
@@ -3749,27 +3749,27 @@
       </c>
       <c r="H52" s="14" t="inlineStr">
         <is>
-          <t>于伟</t>
+          <t>黄睿平</t>
         </is>
       </c>
       <c r="I52" s="14" t="inlineStr">
         <is>
-          <t>15296218518</t>
+          <t>15053584143</t>
         </is>
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>许妍</t>
+          <t>傅玉雪</t>
         </is>
       </c>
       <c r="K52" s="14" t="inlineStr">
         <is>
-          <t>17780670654</t>
+          <t>19918299229</t>
         </is>
       </c>
       <c r="L52" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡小张庄366号</t>
+          <t>河南省-平顶山市-叶县-洪庄杨乡周庄村346号</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>2013年07月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>410422201307194650</t>
+          <t>410422201306239815</t>
         </is>
       </c>
       <c r="G53" s="13" t="n">
@@ -3807,27 +3807,27 @@
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>曾宇浩</t>
+          <t>朱峰</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>19952772217</t>
+          <t>13578447364</t>
         </is>
       </c>
       <c r="J53" s="8" t="inlineStr">
         <is>
-          <t>张燕英</t>
+          <t>萧丽</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>13654868740</t>
+          <t>15076773592</t>
         </is>
       </c>
       <c r="L53" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-仙台镇水郭村293号</t>
+          <t>河南省-平顶山市-叶县-夏李乡杨岭庄村752号</t>
         </is>
       </c>
     </row>
@@ -3847,17 +3847,17 @@
       </c>
       <c r="D54" s="40" t="inlineStr">
         <is>
-          <t>汉</t>
+          <t>满族</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F54" s="13" t="inlineStr">
         <is>
-          <t>410422201305135454</t>
+          <t>41042220130316963X</t>
         </is>
       </c>
       <c r="G54" s="13" t="n">
@@ -3865,27 +3865,27 @@
       </c>
       <c r="H54" s="14" t="inlineStr">
         <is>
-          <t>曹凯</t>
+          <t>吕峰平</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>17741616928</t>
+          <t>18295327877</t>
         </is>
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>马琳琳</t>
+          <t>罗涵悦</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>15947962757</t>
+          <t>17773395004</t>
         </is>
       </c>
       <c r="L54" s="17" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇思城村630号</t>
+          <t>河南省-平顶山市-叶县-龚店乡周庄村904号</t>
         </is>
       </c>
     </row>
@@ -3910,40 +3910,40 @@
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F55" s="13" t="inlineStr">
         <is>
-          <t>410422201209305075</t>
+          <t>410422201301144742</t>
         </is>
       </c>
       <c r="G55" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H55" s="14" t="inlineStr">
         <is>
-          <t>唐凯</t>
+          <t>谢俊</t>
         </is>
       </c>
       <c r="I55" s="14" t="inlineStr">
         <is>
-          <t>15002970213</t>
+          <t>18609835841</t>
         </is>
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>谢怡</t>
+          <t>韩妍</t>
         </is>
       </c>
       <c r="K55" s="14" t="inlineStr">
         <is>
-          <t>13692755719</t>
+          <t>19949912165</t>
         </is>
       </c>
       <c r="L55" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-辛店镇刘庄村376号</t>
+          <t>河南省-平顶山市-叶县-仙台镇杨岭庄村572号</t>
         </is>
       </c>
     </row>
@@ -3968,12 +3968,12 @@
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>2012年09月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F56" s="13" t="inlineStr">
         <is>
-          <t>41042220120914261X</t>
+          <t>410422201211106974</t>
         </is>
       </c>
       <c r="G56" s="13" t="n">
@@ -3981,27 +3981,27 @@
       </c>
       <c r="H56" s="14" t="inlineStr">
         <is>
-          <t>孙然</t>
+          <t>宋豪</t>
         </is>
       </c>
       <c r="I56" s="14" t="inlineStr">
         <is>
-          <t>19914473947</t>
+          <t>13998259526</t>
         </is>
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>胡霞丽</t>
+          <t>吕雪</t>
         </is>
       </c>
       <c r="K56" s="14" t="inlineStr">
         <is>
-          <t>18827155188</t>
+          <t>17788794705</t>
         </is>
       </c>
       <c r="L56" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-常村镇凤岭新村872号</t>
+          <t>河南省-平顶山市-叶县-夏李乡梅湾村427号</t>
         </is>
       </c>
     </row>
@@ -4026,40 +4026,40 @@
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>2012年11月</t>
+          <t>2013年03月</t>
         </is>
       </c>
       <c r="F57" s="14" t="inlineStr">
         <is>
-          <t>410422201211026295</t>
+          <t>410422201303142777</t>
         </is>
       </c>
       <c r="G57" s="14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H57" s="14" t="inlineStr">
         <is>
-          <t>周鹏</t>
+          <t>林磊</t>
         </is>
       </c>
       <c r="I57" s="14" t="inlineStr">
         <is>
-          <t>13558957829</t>
+          <t>13830756263</t>
         </is>
       </c>
       <c r="J57" s="14" t="inlineStr">
         <is>
-          <t>杨丽</t>
+          <t>冯妍</t>
         </is>
       </c>
       <c r="K57" s="14" t="inlineStr">
         <is>
-          <t>17686691251</t>
+          <t>17602838578</t>
         </is>
       </c>
       <c r="L57" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡王庄村697号</t>
+          <t>河南省-平顶山市-叶县-田庄乡杨岭庄村980号</t>
         </is>
       </c>
     </row>
@@ -4084,12 +4084,12 @@
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>2013年06月</t>
+          <t>2013年01月</t>
         </is>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
-          <t>410422201306106461</t>
+          <t>410422201301315903</t>
         </is>
       </c>
       <c r="G58" s="14" t="n">
@@ -4097,27 +4097,27 @@
       </c>
       <c r="H58" s="14" t="inlineStr">
         <is>
-          <t>曾刚</t>
+          <t>马文</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>13968018242</t>
+          <t>17657584419</t>
         </is>
       </c>
       <c r="J58" s="14" t="inlineStr">
         <is>
-          <t>徐琳</t>
+          <t>许佳</t>
         </is>
       </c>
       <c r="K58" s="5" t="inlineStr">
         <is>
-          <t>15258414384</t>
+          <t>18652404157</t>
         </is>
       </c>
       <c r="L58" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-辛店镇凤岭新村630号</t>
+          <t>河南省-平顶山市-叶县-廉村镇蔡庄村766号</t>
         </is>
       </c>
     </row>
@@ -4147,7 +4147,7 @@
       </c>
       <c r="F59" s="14" t="inlineStr">
         <is>
-          <t>410422201211185506</t>
+          <t>410422201211106873</t>
         </is>
       </c>
       <c r="G59" s="14" t="n">
@@ -4155,27 +4155,27 @@
       </c>
       <c r="H59" s="14" t="inlineStr">
         <is>
-          <t>吕宇</t>
+          <t>吕鹏睿</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>13601094396</t>
+          <t>15230165712</t>
         </is>
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>吕娜</t>
+          <t>王曦</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>19944736471</t>
+          <t>15067734540</t>
         </is>
       </c>
       <c r="L59" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡孟庄村162号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡盆杨村668号</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>410422201211138812</t>
+          <t>410422201211293632</t>
         </is>
       </c>
       <c r="G60" s="14" t="n">
@@ -4213,27 +4213,27 @@
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>梁浩</t>
+          <t>孙磊</t>
         </is>
       </c>
       <c r="I60" s="14" t="inlineStr">
         <is>
-          <t>13958815371</t>
+          <t>18672400499</t>
         </is>
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>郭诗娟</t>
+          <t>赵婷晴</t>
         </is>
       </c>
       <c r="K60" s="14" t="inlineStr">
         <is>
-          <t>13646963259</t>
+          <t>17772874315</t>
         </is>
       </c>
       <c r="L60" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-洪庄杨乡杨岭庄村195号</t>
+          <t>河南省-平顶山市-叶县-辛店镇王庄村664号</t>
         </is>
       </c>
     </row>
@@ -4253,45 +4253,45 @@
       </c>
       <c r="D61" s="40" t="inlineStr">
         <is>
-          <t>回族</t>
+          <t>汉</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>2013年05月</t>
+          <t>2012年11月</t>
         </is>
       </c>
       <c r="F61" s="14" t="inlineStr">
         <is>
-          <t>410422201305142995</t>
+          <t>410422201211294142</t>
         </is>
       </c>
       <c r="G61" s="14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H61" s="14" t="inlineStr">
         <is>
-          <t>罗然俊</t>
+          <t>唐阳</t>
         </is>
       </c>
       <c r="I61" s="14" t="inlineStr">
         <is>
-          <t>17773395004</t>
+          <t>13761227530</t>
         </is>
       </c>
       <c r="J61" s="14" t="inlineStr">
         <is>
-          <t>曹萱芳</t>
+          <t>何佳玉</t>
         </is>
       </c>
       <c r="K61" s="14" t="inlineStr">
         <is>
-          <t>13862456506</t>
+          <t>18249904530</t>
         </is>
       </c>
       <c r="L61" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-叶邑镇孙庄村576号</t>
+          <t>河南省-平顶山市-叶县-廉村镇梅湾村477号</t>
         </is>
       </c>
     </row>
@@ -4316,12 +4316,12 @@
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>2013年04月</t>
+          <t>2013年02月</t>
         </is>
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
-          <t>410422201304194359</t>
+          <t>410422201302071638</t>
         </is>
       </c>
       <c r="G62" s="14" t="n">
@@ -4329,27 +4329,27 @@
       </c>
       <c r="H62" s="14" t="inlineStr">
         <is>
-          <t>傅飞</t>
+          <t>黄鑫</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>13821655852</t>
+          <t>15232727956</t>
         </is>
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>胡妍</t>
+          <t>傅萱</t>
         </is>
       </c>
       <c r="K62" s="5" t="inlineStr">
         <is>
-          <t>13600257872</t>
+          <t>15139187851</t>
         </is>
       </c>
       <c r="L62" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-水寨乡刘庄村144号</t>
+          <t>河南省-平顶山市-叶县-马庄回族乡孙庄村115号</t>
         </is>
       </c>
     </row>
@@ -4374,12 +4374,12 @@
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>2013年02月</t>
+          <t>2013年05月</t>
         </is>
       </c>
       <c r="F63" s="14" t="inlineStr">
         <is>
-          <t>410422201302017449</t>
+          <t>410422201305208872</t>
         </is>
       </c>
       <c r="G63" s="14" t="n">
@@ -4387,27 +4387,27 @@
       </c>
       <c r="H63" s="14" t="inlineStr">
         <is>
-          <t>宋轩</t>
+          <t>刘博峰</t>
         </is>
       </c>
       <c r="I63" s="14" t="inlineStr">
         <is>
-          <t>19979470551</t>
+          <t>18890874064</t>
         </is>
       </c>
       <c r="J63" s="14" t="inlineStr">
         <is>
-          <t>冯雪</t>
+          <t>王梅</t>
         </is>
       </c>
       <c r="K63" s="14" t="inlineStr">
         <is>
-          <t>13597499309</t>
+          <t>13665180170</t>
         </is>
       </c>
       <c r="L63" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龚店乡老鸦张村537号</t>
+          <t>河南省-平顶山市-叶县-常村镇李庄村185号</t>
         </is>
       </c>
     </row>
@@ -4432,12 +4432,12 @@
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>2013年03月</t>
+          <t>2013年06月</t>
         </is>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>410422201303314053</t>
+          <t>410422201306037080</t>
         </is>
       </c>
       <c r="G64" s="14" t="n">
@@ -4445,27 +4445,27 @@
       </c>
       <c r="H64" s="14" t="inlineStr">
         <is>
-          <t>朱峰</t>
+          <t>邓明</t>
         </is>
       </c>
       <c r="I64" s="14" t="inlineStr">
         <is>
-          <t>17602838578</t>
+          <t>15200478686</t>
         </is>
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>韩琳</t>
+          <t>高红</t>
         </is>
       </c>
       <c r="K64" s="14" t="inlineStr">
         <is>
-          <t>18885854973</t>
+          <t>13943106903</t>
         </is>
       </c>
       <c r="L64" s="14" t="inlineStr">
         <is>
-          <t>河南省-平顶山市-叶县-龙泉乡蔡庄村572号</t>
+          <t>河南省-平顶山市-叶县-龙泉乡盆杨村104号</t>
         </is>
       </c>
     </row>

</xml_diff>